<commit_message>
feat(grading): align S06 scoring with the revised evaluation criteria
</commit_message>
<xml_diff>
--- a/skills/04-excel-grading/assets/01_template/S06_excel_scoring_criteria_v1.xlsx
+++ b/skills/04-excel-grading/assets/01_template/S06_excel_scoring_criteria_v1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\【github_rjsiao】\my-ai-skills\skills\04-excel-grading\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\【github_rjsiao】\my-ai-skills\skills\04-excel-grading\assets\01_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -45,28 +45,18 @@
     <t>1.1-作答狀態初步判斷。</t>
   </si>
   <si>
-    <t>使用【薪資】活頁的A1:J13資料，成功建立樞紐表，檔案中的樞紐表與原始資料可能在不同活頁，但要先排除【考題】活頁的範例答案。若沒有任何樞紐表，「考題1.薪資」所有小項都給0分。</t>
-  </si>
-  <si>
     <t>【高】可用 openpyxl 讀取工作表的樞紐表物件（ws._pivots／xl/pivotTables 底下的 XML），判斷【薪資】活頁是否成功建立樞紐表，並依 cacheId 對應之來源範圍排除【考題】活頁本身的範例樞紐表。</t>
   </si>
   <si>
     <t>1.2-欄列標籤選取。</t>
   </si>
   <si>
-    <t>樞紐表的「欄標籤」放在橫軸、只篩選出業務，「列標籤」放在縱軸、要同時有男、女。「欄標籤」若是同時列出「業務、會計、門市」只給一半分數，完全不是這三個其中一個的給0分；「列標籤」沒有放「男、女」的給0分。
-【折衷微調】若「欄標籤」完整顯示三個部門（業務、會計、門市）且「列標籤」正確呈現男、女，屬於更完整的樞紐分析呈現方式，建議仍給予滿分，不再視為錯誤。</t>
-  </si>
-  <si>
     <t>【中】openpyxl 可讀出 pivotFields 的 axis 屬性（axisRow／axisCol）判斷「性別」「部門」何者置於列／欄；但要進一步確認欄標籤是否僅顯示「業務」單一項目，需額外解析 pivotCacheDefinition／pivotCacheRecords 的共用項目清單與 hidden(h) 標記，屬於 openpyxl 未直接封裝的底層 XML 判讀，需自行寫程式解析，但仍可行。</t>
   </si>
   <si>
     <t>1.3-樞紐值的彙總方式。</t>
   </si>
   <si>
-    <t>樞紐表的「值欄位」設定是平均值；若是「加總」，只給一半配分。</t>
-  </si>
-  <si>
     <t>【高】樞紐表 dataFields 物件有 subtotal 屬性（'average'／'sum'…），可直接讀取判斷彙總方式。</t>
   </si>
   <si>
@@ -94,9 +84,6 @@
     <t>2.1-凍結窗格設定。</t>
   </si>
   <si>
-    <t>在【成績】活頁，凍結窗格設在B3，讓分數以外的科目列、姓名欄固定不動，不因滑鼠滾動而移動。若科目列(第2列)、姓名欄位(第A欄)兩者都有成功固定的話，各給一半的配分。</t>
-  </si>
-  <si>
     <t>【高】openpyxl 可直接讀取 ws.freeze_panes（如 'B3'），並可判斷是否同時凍結列與欄，或僅凍結其一（如 'A3' 或 'B1'），對應給予半分或滿分。</t>
   </si>
   <si>
@@ -115,18 +102,12 @@
     <t>2.5-資料格線樣式設計。</t>
   </si>
   <si>
-    <t>在【成績】活頁的A1:G16範圍中，使用框線區隔。</t>
-  </si>
-  <si>
     <t>【中】openpyxl 可讀取每個儲存格的 border 屬性（top／bottom／left／right 樣式），需逐格檢查 A1:G16 範圍是否皆有框線設定，屬可行但較繁瑣的迴圈比對工作。</t>
   </si>
   <si>
     <t>2.6-處理有問題儲存格。(額外加分)</t>
   </si>
   <si>
-    <t>在【成績】活頁的G16單格中，未使用任何Excel公式。</t>
-  </si>
-  <si>
     <t>【高】可直接檢查 G16 儲存格的 data_type 是否為 'f'（公式），或內容是否為 None／純數值，判斷簡單明確。</t>
   </si>
   <si>
@@ -140,9 +121,6 @@
   </si>
   <si>
     <t>3.2-圖表座標軸設定。</t>
-  </si>
-  <si>
-    <t>在【車輛銷售】的長條圖或直方圖中，水平座標軸只有「福特、賓士、裕隆、三菱」，多出的或缺項皆不可，四個類別全部都顯示才能給三分之一配分。再三分之一配分，用在數量的「最大值」設為2000、「主要單位」500的這兩項，全對才給分。最後三分之一配分，用在主要格線格式無線條。</t>
   </si>
   <si>
     <t>【高】類別項目可讀 cat.strRef 快取字串清單（福特/賓士/裕隆/三菱）；數值軸最大值／主要單位可讀 y_axis.scaling.max／y_axis.majorUnit；主要格線是否無線條可檢查 y_axis.majorGridlines 是否為 None 或其線條屬性 noFill=True，皆為 openpyxl 可直接存取的屬性。</t>
@@ -179,47 +157,77 @@
     <t>4.2-圖表座標設定。</t>
   </si>
   <si>
-    <t>在【武將能力】的雷達圖，水平座標軸只有「趙雲、周瑜、程遠志、劉禪」，圖例項目只有「統帥、武力、致力、政治、魅力」，多出的或缺項皆不可，水平座標軸、圖例項目都全部都顯示才能給完整配分，否則給0分。圖例位置及配色都不限制。
-【補充】可拆解為「水平座標軸(統帥/武力/智力/政治/魅力)5分」＋「圖例項目(趙雲/周瑜/程遠志/劉禪)5分」，兩者皆全對才給滿分10分，任一缺漏則該部分給0分。</t>
-  </si>
-  <si>
     <t>【高】可讀取雷達圖 cat.strRef 快取字串（統帥/武力/智力/政治/魅力）與各數列 tx.strRef（趙雲/周瑜/程遠志/劉禪），確認類別與圖例項目是否完整、有無缺漏。</t>
   </si>
   <si>
     <t>4.3-圖表資訊美化。(額外加分)</t>
   </si>
   <si>
+    <t>【高】圖表標題同3.4可讀 chart.title；「含資料點標記」可直接讀 chart.type 屬性（'marker'／'standard'／'filled'）判斷是否為含標記樣式的雷達圖，判斷邏輯簡單明確。</t>
+  </si>
+  <si>
+    <t>在【武將能力】有建立一個雷達圖，若沒有「動態」的雷達圖，「考題4.武將能力」所有小項都給0分。若有多張圖表，只查看取得動態資料的雷達圖，其餘圖表皆忽略不看。若第A欄及第2列的任一原始資料有改動，「考題4.武將能力」的小項皆不予計分。原題目【武將能力】D2「程遠志」尾端含一個看不見的Tab字元；學員若只刪除這類前後空白字元、畫面顯示不變，不視為原始資料改動。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.4-排序與篩選設定。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【成績】活頁，用AVG函式算出每一列的「個人平均」，完整放在G3:G15，得一半配分；再用AVG函式算出的每一欄的「班平均」，每個計算結果都只保留到整數位，再得另一半配分。如果「班平均」的計算結果不在最後一列(第16列)，請先找A欄是「班平均」的那一列。「班平均」須使用AVERAGE函式；以表格合計列的SUBTOTAL(101,…)或其他函式取代AVERAGE者，「班平均」這一半給0分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2.2-標頭跨欄置中設定。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>在【武將能力】的雷達圖，達成以下圖表設計，每項可以加分3分：(1) 加上圖表標題，如「武將各項能力表」。(2) 使用含資料點標記的雷達圖。</t>
-  </si>
-  <si>
-    <t>【高】圖表標題同3.4可讀 chart.title；「含資料點標記」可直接讀 chart.type 屬性（'marker'／'standard'／'filled'）判斷是否為含標記樣式的雷達圖，判斷邏輯簡單明確。</t>
-  </si>
-  <si>
-    <t>在【武將能力】有建立一個雷達圖，若沒有「動態」的雷達圖，「考題4.武將能力」所有小項都給0分。若有多張圖表，只查看取得動態資料的雷達圖，其餘圖表皆忽略不看。若第A欄及第2列的任一原始資料有改動，「考題4.武將能力」的小項皆不予計分。原題目【武將能力】D2「程遠志」尾端含一個看不見的Tab字元；學員若只刪除這類前後空白字元、畫面顯示不變，不視為原始資料改動。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>在【車輛銷售】有建立一個群組直條圖，若沒有「動態」的直條圖，「考題3.車輛銷售」所有小項都給0分。若有多張圖表，只查看取得動態資料的長條圖或直方圖，其餘圖表皆忽略不看。若第A欄及第2列的任一原始資料有改動，「考題3.車輛銷售」的小項皆不予計分。「立體群組直條圖」（3-D群組直條圖）視同群組直條圖，照常給分。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2.4-排序與篩選設定。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>在【成績】活頁，用AVG函式算出每一列的「個人平均」，完整放在G3:G15，得一半配分；再用AVG函式算出的每一欄的「班平均」，每個計算結果都只保留到整數位，再得另一半配分。如果「班平均」的計算結果不在最後一列(第16列)，請先找A欄是「班平均」的那一列。「班平均」須使用AVERAGE函式；以表格合計列的SUBTOTAL(101,…)或其他函式取代AVERAGE者，「班平均」這一半給0分。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>在【成績】活頁，檢查「個人平均」G3:G15是否由大到小排序，成功得5分；再看G2是否以「數字篩選」設定「大於70」或「大於或等於70」，最終只留下9列資料（7位學生加上班平均），成功得5分。以勾選數值清單方式篩選（即使結果相同），或篩選條件設在「個人平均」以外的欄位，篩選這5分給0分。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2.2-標頭跨欄置中設定。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>在【成績】活頁，對A1:G1設定跨欄置中（或合併後置中）得2分，範圍須剛好是A1:G1，超出範圍（例如A1:H1）不給這2分；跨欄置中後標題仍維持「經濟甲班 期中考成績表」，再得2分。完全沒有設定跨欄置中或合併者，本項0分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【成績】活頁，凍結窗格設在B3，讓分數以外的科目列、姓名欄固定不動，不因滑鼠滾動而移動。若科目列(第2列)、姓名欄位(第A欄)兩者都有成功固定的話，各給一半的配分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【成績】活頁的A1:G16範圍中，使用框線區隔。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【車輛銷售】的長條圖或直方圖中，水平座標軸只有「福特、賓士、裕隆、三菱」，多出的或缺項皆不可，四個類別全部都顯示才能給三分之一配分。再三分之一配分，用在數量的「最大值」設為2000、「主要單位」500的這兩項，全對才給分。最後三分之一配分，用在主要格線格式無線條。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【成績】活頁，檢查「個人平均」G3:G15是否由大到小排序，成功得5分；再看G2是否以「數字篩選」設定「大於70」或「大於或等於70」，最終只留下9列資料（8位學生加上班平均），成功得5分。以勾選數值清單方式篩選（即使結果相同），或篩選條件設在「個人平均」以外的欄位，篩選這5分給0分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>使用【薪資】活頁的A1:J13資料，成功建立樞紐表，檔案中的樞紐表與原始資料可能在不同活頁，但要先排除【考題】活頁的範例答案，允許另外建立有前後綴活頁名稱（如【1.薪資】【薪資_ans】）。若沒有任何樞紐表，「考題1.薪資」所有小項都給0分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【成績】活頁的G16單格中，未使用任何Excel公式，且數值、文字也不可填。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【車輛銷售】有建立一個群組直條圖，若沒有「動態」的直條圖，「考題3.車輛銷售」所有小項都給0分。若有多張圖表，只查看取得動態資料的長條圖或直方圖，其餘圖表皆忽略不看。若第A欄及第2列的任一原始資料有改動，「考題3.車輛銷售」的小項皆不予計分。「立體群組直條圖」（3-D群組直條圖）、「直方圖」都視同群組直條圖，照常給分；只限長條圖、直條圖、直方圖，其餘圖表皆不給分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【成績】活頁，對A1:G1設定，同時有完成合併後置中(不可超出範圍)得2分，範圍須剛好是A1:G1；該儲存格的標題是「經濟甲班 期中考成績表」，再得2分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>樞紐表的「欄標籤」放在橫軸、只篩選出業務，「列標籤」放在縱軸、要同時有男、女。「欄標籤」若不是「業務、會計、門市」任何一個的，請直接給0分；「列標籤」不是「男、女」的也直接給0分。「欄標籤」不是只留下「業務」扣5分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【武將能力】的雷達圖，水平座標軸只有「統帥、武力、智力、政治、魅力」，圖例項目只有「趙雲、周瑜、程遠志、劉禪」，多出的或缺項皆不可，正確顯示的話水平座標軸、圖例項目各自得5分。圖例位置及配色都不限制。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>樞紐表的「值欄位」設定是平均值；若是「加總」，只給一半配分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -613,7 +621,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="63" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -621,7 +629,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="D2" s="3">
         <v>5</v>
@@ -630,18 +638,18 @@
         <v>0</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="D3" s="3">
         <v>10</v>
@@ -650,18 +658,18 @@
         <v>0</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>14</v>
+        <v>63</v>
       </c>
       <c r="D4" s="3">
         <v>10</v>
@@ -670,18 +678,18 @@
         <v>0</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D5" s="3">
         <v>5</v>
@@ -690,18 +698,18 @@
         <v>0</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D6" s="3">
         <v>0</v>
@@ -710,18 +718,18 @@
         <v>6</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="D7" s="3">
         <v>4</v>
@@ -730,18 +738,18 @@
         <v>0</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="63" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D8" s="3">
         <v>4</v>
@@ -750,18 +758,18 @@
         <v>0</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D9" s="3">
         <v>9</v>
@@ -770,18 +778,18 @@
         <v>0</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D10" s="3">
         <v>10</v>
@@ -790,18 +798,18 @@
         <v>0</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="D11" s="3">
         <v>3</v>
@@ -810,18 +818,18 @@
         <v>0</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="D12" s="3">
         <v>0</v>
@@ -830,18 +838,18 @@
         <v>3</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D13" s="3">
         <v>5</v>
@@ -850,18 +858,18 @@
         <v>0</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D14" s="3">
         <v>15</v>
@@ -870,18 +878,18 @@
         <v>0</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>43</v>
       </c>
       <c r="D15" s="3">
         <v>5</v>
@@ -890,18 +898,18 @@
         <v>0</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="D16" s="3">
         <v>0</v>
@@ -910,18 +918,18 @@
         <v>9</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>57</v>
       </c>
       <c r="D17" s="3">
         <v>5</v>
@@ -930,18 +938,18 @@
         <v>0</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="D18" s="3">
         <v>10</v>
@@ -950,18 +958,18 @@
         <v>0</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D19" s="3">
         <v>0</v>
@@ -970,7 +978,7 @@
         <v>6</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(grading): tighten rubric matching to exact ranges
</commit_message>
<xml_diff>
--- a/skills/04-excel-grading/assets/01_template/S06_excel_scoring_criteria_v1.xlsx
+++ b/skills/04-excel-grading/assets/01_template/S06_excel_scoring_criteria_v1.xlsx
@@ -166,10 +166,6 @@
     <t>【高】圖表標題同3.4可讀 chart.title；「含資料點標記」可直接讀 chart.type 屬性（'marker'／'standard'／'filled'）判斷是否為含標記樣式的雷達圖，判斷邏輯簡單明確。</t>
   </si>
   <si>
-    <t>在【武將能力】有建立一個雷達圖，若沒有「動態」的雷達圖，「考題4.武將能力」所有小項都給0分。若有多張圖表，只查看取得動態資料的雷達圖，其餘圖表皆忽略不看。若第A欄及第2列的任一原始資料有改動，「考題4.武將能力」的小項皆不予計分。原題目【武將能力】D2「程遠志」尾端含一個看不見的Tab字元；學員若只刪除這類前後空白字元、畫面顯示不變，不視為原始資料改動。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>2.4-排序與篩選設定。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -202,31 +198,35 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>使用【薪資】活頁的A1:J13資料，成功建立樞紐表，檔案中的樞紐表與原始資料可能在不同活頁，但要先排除【考題】活頁的範例答案，允許另外建立有前後綴活頁名稱（如【1.薪資】【薪資_ans】）。若沒有任何樞紐表，「考題1.薪資」所有小項都給0分。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>在【成績】活頁的G16單格中，未使用任何Excel公式，且數值、文字也不可填。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>在【車輛銷售】有建立一個群組直條圖，若沒有「動態」的直條圖，「考題3.車輛銷售」所有小項都給0分。若有多張圖表，只查看取得動態資料的長條圖或直方圖，其餘圖表皆忽略不看。若第A欄及第2列的任一原始資料有改動，「考題3.車輛銷售」的小項皆不予計分。「立體群組直條圖」（3-D群組直條圖）、「直方圖」都視同群組直條圖，照常給分；只限長條圖、直條圖、直方圖，其餘圖表皆不給分。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>在【成績】活頁，對A1:G1設定，同時有完成合併後置中(不可超出範圍)得2分，範圍須剛好是A1:G1；該儲存格的標題是「經濟甲班 期中考成績表」，再得2分。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>樞紐表的「欄標籤」放在橫軸、只篩選出業務，「列標籤」放在縱軸、要同時有男、女。「欄標籤」若不是「業務、會計、門市」任何一個的，請直接給0分；「列標籤」不是「男、女」的也直接給0分。「欄標籤」不是只留下「業務」扣5分。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>在【武將能力】的雷達圖，水平座標軸只有「統帥、武力、智力、政治、魅力」，圖例項目只有「趙雲、周瑜、程遠志、劉禪」，多出的或缺項皆不可，正確顯示的話水平座標軸、圖例項目各自得5分。圖例位置及配色都不限制。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>樞紐表的「值欄位」設定是平均值；若是「加總」，只給一半配分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>使用【薪資】活頁的A1:J13資料，成功建立樞紐表，檔案中的樞紐表與原始資料可能在不同活頁，但要先排除【考題】活頁的範例答案，允許另外建立有前後綴活頁名稱（如【1.薪資】【薪資_ans】）。若沒有任何樞紐表，「考題1.薪資」所有小項都給0分。未使用【薪資】活頁的A1:J13資料製作樞紐表者，「考題1.薪資」所有小項都給0分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>樞紐表的「欄標籤」放在橫軸、只篩選出業務，「列標籤」放在縱軸、要同時有男、女。「欄標籤」若不是「業務、會計、門市」任何一個的，或者「列標籤」不是「男、女」的，兩個都直接給0分。「欄標籤」不是只留下「業務」扣5分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【車輛銷售】有建立一個群組直條圖，若沒有「動態」的直條圖，「考題3.車輛銷售」所有小項都給0分。若有多張圖表，只查看取得動態資料的長條圖或直方圖，其餘圖表皆忽略不看。若第A欄(A2:A6)及第2列(A2:E2)的任一原始資料有改動，「考題3.車輛銷售」的小項皆不予計分。「立體群組直條圖」（3-D群組直條圖）、「直方圖」都視同群組直條圖，照常給分；只限長條圖、直條圖、直方圖，其餘圖表皆不給分。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在【武將能力】有建立一個雷達圖，若沒有「動態」的雷達圖，「考題4.武將能力」所有小項都給0分。若有多張圖表，只查看取得動態資料的雷達圖，其餘圖表皆忽略不看。若第A欄(A2:A7)及第2列(A2:E2)的任一原始資料有改動，「考題4.武將能力」的小項皆不予計分。原題目【武將能力】D2「程遠志」尾端含一個看不見的Tab字元；學員若只刪除這類前後空白字元、畫面顯示不變，不視為原始資料改動。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -629,7 +629,7 @@
         <v>7</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D2" s="3">
         <v>5</v>
@@ -669,7 +669,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D4" s="3">
         <v>10</v>
@@ -729,7 +729,7 @@
         <v>20</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D7" s="3">
         <v>4</v>
@@ -746,10 +746,10 @@
         <v>19</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D8" s="3">
         <v>4</v>
@@ -769,7 +769,7 @@
         <v>23</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D9" s="3">
         <v>9</v>
@@ -786,10 +786,10 @@
         <v>19</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D10" s="3">
         <v>10</v>
@@ -809,7 +809,7 @@
         <v>26</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D11" s="3">
         <v>3</v>
@@ -829,7 +829,7 @@
         <v>28</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D12" s="3">
         <v>0</v>
@@ -849,7 +849,7 @@
         <v>31</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D13" s="3">
         <v>5</v>
@@ -869,7 +869,7 @@
         <v>33</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D14" s="3">
         <v>15</v>
@@ -929,7 +929,7 @@
         <v>42</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="D17" s="3">
         <v>5</v>
@@ -949,7 +949,7 @@
         <v>44</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D18" s="3">
         <v>10</v>
@@ -969,7 +969,7 @@
         <v>46</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D19" s="3">
         <v>0</v>
@@ -984,6 +984,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>